<commit_message>
Improve ISIC classifier + make report schema-independent
- Weight keyword hits in the project title above body-text hits.
- Add decisive title rule mapping population/housing censuses and IPUMS
  subsets to Public administration (84), excluding sector-specific censuses.
- Derive the repository list in the PDF report from PROJECTS.repository_id
  (and repository_url for names) instead of the removed REPOSITORIES table,
  so Part 2 runs against the cleaned-up Part 1 schema.
</commit_message>
<xml_diff>
--- a/23080363-sq26-classification.xlsx
+++ b/23080363-sq26-classification.xlsx
@@ -484,12 +484,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -568,12 +568,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -596,12 +596,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -624,12 +624,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -652,12 +652,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -680,12 +680,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -708,12 +708,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -736,12 +736,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -764,12 +764,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -792,12 +792,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Employment activities</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -820,12 +820,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -848,12 +848,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -876,12 +876,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -904,12 +904,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -932,12 +932,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -960,12 +960,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -988,12 +988,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1016,12 +1016,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1044,12 +1044,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1072,12 +1072,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1100,12 +1100,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1128,12 +1128,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Employment activities</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -1184,12 +1184,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1240,12 +1240,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1268,12 +1268,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1296,12 +1296,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1324,12 +1324,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -1352,12 +1352,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -1380,12 +1380,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -1408,12 +1408,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -1436,12 +1436,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Crop and animal production, hunting and related service activities</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -1464,12 +1464,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -1492,12 +1492,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -1520,12 +1520,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -1548,12 +1548,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -1576,12 +1576,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -1604,12 +1604,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -1632,12 +1632,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -1660,12 +1660,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -1688,12 +1688,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -1716,12 +1716,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -1744,12 +1744,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -1772,12 +1772,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -1800,12 +1800,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -1828,12 +1828,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -1856,12 +1856,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -1884,12 +1884,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -1912,12 +1912,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -1940,12 +1940,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -1968,12 +1968,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -1996,12 +1996,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -2024,12 +2024,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -2052,12 +2052,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F58" t="n">
@@ -2080,12 +2080,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -2108,12 +2108,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F60" t="n">
@@ -2136,12 +2136,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -2164,12 +2164,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F62" t="n">
@@ -2192,12 +2192,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -2220,12 +2220,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -2248,12 +2248,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -2276,12 +2276,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -2304,12 +2304,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Crop and animal production, hunting and related service activities</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -2332,12 +2332,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -2360,12 +2360,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -2388,12 +2388,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -2416,12 +2416,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -2444,12 +2444,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -2472,12 +2472,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -2500,12 +2500,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -2528,12 +2528,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -2556,12 +2556,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -2584,12 +2584,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F77" t="n">
@@ -2612,12 +2612,12 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F78" t="n">
@@ -2640,12 +2640,12 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -2668,12 +2668,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -2696,12 +2696,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -2724,12 +2724,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -2752,12 +2752,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -2780,12 +2780,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F84" t="n">
@@ -2808,12 +2808,12 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -2836,12 +2836,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F86" t="n">
@@ -2864,12 +2864,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -2892,12 +2892,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F88" t="n">
@@ -2920,12 +2920,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F89" t="n">
@@ -2948,12 +2948,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -2976,12 +2976,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F91" t="n">
@@ -3004,12 +3004,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -3032,12 +3032,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -3060,12 +3060,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -3088,12 +3088,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -3116,12 +3116,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -3144,12 +3144,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F97" t="n">
@@ -3172,12 +3172,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -3200,12 +3200,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Employment activities</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -3228,12 +3228,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -3256,12 +3256,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -3284,12 +3284,12 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -3312,12 +3312,12 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -3340,12 +3340,12 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -3368,12 +3368,12 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F105" t="n">
@@ -3396,12 +3396,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F106" t="n">
@@ -3424,12 +3424,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -3452,12 +3452,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F108" t="n">
@@ -3480,12 +3480,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F109" t="n">
@@ -3508,12 +3508,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F110" t="n">
@@ -3536,12 +3536,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F111" t="n">
@@ -3588,12 +3588,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F113" t="n">
@@ -4280,12 +4280,12 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Social work activities without accommodation</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F138" t="n">
@@ -4308,12 +4308,12 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Social work activities without accommodation</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F139" t="n">
@@ -12004,12 +12004,12 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E414" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F414" t="n">
@@ -12032,12 +12032,12 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E415" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F415" t="n">
@@ -12060,12 +12060,12 @@
       </c>
       <c r="D416" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E416" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F416" t="n">
@@ -12088,12 +12088,12 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E417" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F417" t="n">
@@ -12116,12 +12116,12 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E418" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F418" t="n">
@@ -12144,12 +12144,12 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E419" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F419" t="n">
@@ -12172,12 +12172,12 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E420" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F420" t="n">
@@ -12200,7 +12200,7 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E421" t="inlineStr">
@@ -12228,12 +12228,12 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E422" t="inlineStr">
-        <is>
-          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F422" t="n">
@@ -12256,7 +12256,7 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Forestry and logging</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E423" t="inlineStr">
@@ -12284,12 +12284,12 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E424" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F424" t="n">
@@ -12312,12 +12312,12 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E425" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F425" t="n">
@@ -12340,12 +12340,12 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E426" t="inlineStr">
-        <is>
-          <t>Fishing and aquaculture</t>
         </is>
       </c>
       <c r="F426" t="n">
@@ -12368,12 +12368,12 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E427" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F427" t="n">
@@ -12396,12 +12396,12 @@
       </c>
       <c r="D428" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E428" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F428" t="n">
@@ -12424,12 +12424,12 @@
       </c>
       <c r="D429" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E429" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F429" t="n">
@@ -12480,12 +12480,12 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E431" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F431" t="n">
@@ -12508,12 +12508,12 @@
       </c>
       <c r="D432" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E432" t="inlineStr">
-        <is>
-          <t>Fishing and aquaculture</t>
         </is>
       </c>
       <c r="F432" t="n">
@@ -12536,12 +12536,12 @@
       </c>
       <c r="D433" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E433" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F433" t="n">
@@ -12564,7 +12564,7 @@
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Fishing and aquaculture</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E434" t="inlineStr">
@@ -12592,12 +12592,12 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E435" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F435" t="n">
@@ -12620,12 +12620,12 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E436" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F436" t="n">
@@ -12648,12 +12648,12 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E437" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F437" t="n">
@@ -12676,12 +12676,12 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E438" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F438" t="n">
@@ -12704,12 +12704,12 @@
       </c>
       <c r="D439" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E439" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F439" t="n">
@@ -12732,12 +12732,12 @@
       </c>
       <c r="D440" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E440" t="inlineStr">
-        <is>
-          <t>Fishing and aquaculture</t>
         </is>
       </c>
       <c r="F440" t="n">
@@ -12760,12 +12760,12 @@
       </c>
       <c r="D441" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E441" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F441" t="n">
@@ -12788,12 +12788,12 @@
       </c>
       <c r="D442" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E442" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F442" t="n">
@@ -12816,12 +12816,12 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E443" t="inlineStr">
-        <is>
-          <t>Employment activities</t>
         </is>
       </c>
       <c r="F443" t="n">
@@ -12844,12 +12844,12 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E444" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F444" t="n">
@@ -12872,12 +12872,12 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E445" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F445" t="n">
@@ -12900,12 +12900,12 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E446" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F446" t="n">
@@ -12928,12 +12928,12 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E447" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F447" t="n">
@@ -12956,12 +12956,12 @@
       </c>
       <c r="D448" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E448" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F448" t="n">
@@ -13213,7 +13213,7 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F457" t="n">
@@ -14184,12 +14184,12 @@
       </c>
       <c r="D492" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E492" t="inlineStr">
-        <is>
-          <t>Employment activities</t>
         </is>
       </c>
       <c r="F492" t="n">
@@ -14217,7 +14217,7 @@
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Crop and animal production, hunting and related service activities</t>
         </is>
       </c>
       <c r="F493" t="n">
@@ -14240,12 +14240,12 @@
       </c>
       <c r="D494" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E494" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F494" t="n">
@@ -14268,12 +14268,12 @@
       </c>
       <c r="D495" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E495" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F495" t="n">
@@ -14296,12 +14296,12 @@
       </c>
       <c r="D496" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E496" t="inlineStr">
-        <is>
-          <t>Real estate activities</t>
         </is>
       </c>
       <c r="F496" t="n">
@@ -14324,12 +14324,12 @@
       </c>
       <c r="D497" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E497" t="inlineStr">
-        <is>
-          <t>Fishing and aquaculture</t>
         </is>
       </c>
       <c r="F497" t="n">
@@ -14352,12 +14352,12 @@
       </c>
       <c r="D498" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E498" t="inlineStr">
-        <is>
-          <t>Employment activities</t>
         </is>
       </c>
       <c r="F498" t="n">
@@ -14380,12 +14380,12 @@
       </c>
       <c r="D499" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E499" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F499" t="n">
@@ -14408,12 +14408,12 @@
       </c>
       <c r="D500" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E500" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F500" t="n">
@@ -14436,12 +14436,12 @@
       </c>
       <c r="D501" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
           <t>Crop and animal production, hunting and related service activities</t>
-        </is>
-      </c>
-      <c r="E501" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F501" t="n">
@@ -15140,12 +15140,12 @@
       </c>
       <c r="D535" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E535" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F535" t="n">
@@ -15420,12 +15420,12 @@
       </c>
       <c r="D545" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F545" t="n">
@@ -16344,12 +16344,12 @@
       </c>
       <c r="D578" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F578" t="n">
@@ -16540,12 +16540,12 @@
       </c>
       <c r="D585" t="inlineStr">
         <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
           <t>Scientific research and development</t>
-        </is>
-      </c>
-      <c r="E585" t="inlineStr">
-        <is>
-          <t>Education</t>
         </is>
       </c>
       <c r="F585" t="n">
@@ -16904,12 +16904,12 @@
       </c>
       <c r="D598" t="inlineStr">
         <is>
+          <t>Social work activities without accommodation</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
           <t>Employment activities</t>
-        </is>
-      </c>
-      <c r="E598" t="inlineStr">
-        <is>
-          <t>Human health activities</t>
         </is>
       </c>
       <c r="F598" t="n">
@@ -17105,7 +17105,7 @@
       </c>
       <c r="E605" t="inlineStr">
         <is>
-          <t>Social work activities without accommodation</t>
+          <t>Scientific research and development</t>
         </is>
       </c>
       <c r="F605" t="n">
@@ -19760,12 +19760,12 @@
       </c>
       <c r="D700" t="inlineStr">
         <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
           <t>Employment activities</t>
-        </is>
-      </c>
-      <c r="E700" t="inlineStr">
-        <is>
-          <t>Education</t>
         </is>
       </c>
       <c r="F700" t="n">
@@ -19905,7 +19905,7 @@
       </c>
       <c r="E705" t="inlineStr">
         <is>
-          <t>Employment activities</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="F705" t="n">
@@ -20768,12 +20768,12 @@
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F736" t="n">
@@ -20829,7 +20829,7 @@
       </c>
       <c r="E738" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F738" t="n">
@@ -20908,12 +20908,12 @@
       </c>
       <c r="D741" t="inlineStr">
         <is>
+          <t>Arts creation and performing arts activities</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E741" t="inlineStr">
-        <is>
-          <t>Human health activities</t>
         </is>
       </c>
       <c r="F741" t="n">
@@ -21888,12 +21888,12 @@
       </c>
       <c r="D776" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E776" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F776" t="n">
@@ -22224,12 +22224,12 @@
       </c>
       <c r="D788" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E788" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F788" t="n">
@@ -22476,12 +22476,12 @@
       </c>
       <c r="D797" t="inlineStr">
         <is>
+          <t>Social work activities without accommodation</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E797" t="inlineStr">
-        <is>
-          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F797" t="n">
@@ -22845,7 +22845,7 @@
       </c>
       <c r="E810" t="inlineStr">
         <is>
-          <t>Social work activities without accommodation</t>
+          <t>Library, archives, museum and other cultural activities</t>
         </is>
       </c>
       <c r="F810" t="n">
@@ -23596,12 +23596,12 @@
       </c>
       <c r="D837" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E837" t="inlineStr">
-        <is>
-          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F837" t="n">
@@ -23680,12 +23680,12 @@
       </c>
       <c r="D840" t="inlineStr">
         <is>
+          <t>Human health activities</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E840" t="inlineStr">
-        <is>
-          <t>Human health activities</t>
         </is>
       </c>
       <c r="F840" t="n">
@@ -24100,12 +24100,12 @@
       </c>
       <c r="D855" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E855" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F855" t="n">

</xml_diff>

<commit_message>
Generate classification report outputs
</commit_message>
<xml_diff>
--- a/23080363-sq26-classification.xlsx
+++ b/23080363-sq26-classification.xlsx
@@ -15074,26 +15074,26 @@
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>QD_PROJECT</t>
+          <t>QDA_PROJECT</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>Replication data for: Designing and Analyzing Randomized Experiments: Application to a Japanese Election Survey Experiment</t>
+          <t>Peoria GIS Data, 2003</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="E533" t="inlineStr">
         <is>
-          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>Library, archives, museum and other cultural activities</t>
         </is>
       </c>
       <c r="F533" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="534">
@@ -15107,7 +15107,7 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>Election Results in Benin,1991-2001</t>
+          <t>Replication data for: Designing and Analyzing Randomized Experiments: Application to a Japanese Election Survey Experiment</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
@@ -15121,7 +15121,7 @@
         </is>
       </c>
       <c r="F534" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
     </row>
     <row r="535">
@@ -15135,7 +15135,7 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>Voices from the Pagan Census: A National Survey of Witches and Neo-Pagans in the United States, 1993-1995</t>
+          <t>Election Results in Benin,1991-2001</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
@@ -15145,11 +15145,11 @@
       </c>
       <c r="E535" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F535" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="536">
@@ -15163,21 +15163,21 @@
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>Territorial Change, 1816-2000 (v3.0)</t>
+          <t>Voices from the Pagan Census: A National Survey of Witches and Neo-Pagans in the United States, 1993-1995</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
         <is>
+          <t>Public administration and defence; compulsory social security</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E536" t="inlineStr">
-        <is>
-          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
-        </is>
-      </c>
       <c r="F536" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="537">
@@ -15191,21 +15191,21 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>Violence Data from other Sources</t>
+          <t>Territorial Change, 1816-2000 (v3.0)</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>Social work activities without accommodation</t>
+          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F537" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="538">
@@ -15219,21 +15219,21 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>Tufts Medical School Alumni, 1980</t>
+          <t>Violence Data from other Sources</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E538" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F538" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="539">
@@ -15247,21 +15247,21 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>Replication data for: Chinese Warfare and Politics in the Ancient East Asian International System, ca. 2700 B.C. to 722 B.C.</t>
+          <t>Tufts Medical School Alumni, 1980</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
         <is>
-          <t>Activities of advertising, market research and public relations</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="E539" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="F539" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="540">
@@ -15275,21 +15275,21 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>Replication data for: The Constraining Power of International Treaties: Theory and Methods</t>
+          <t>Replication data for: Chinese Warfare and Politics in the Ancient East Asian International System, ca. 2700 B.C. to 722 B.C.</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Activities of advertising, market research and public relations</t>
         </is>
       </c>
       <c r="E540" t="inlineStr">
         <is>
-          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F540" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
     </row>
     <row r="541">
@@ -15303,21 +15303,21 @@
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>The National Merit Twin Study</t>
+          <t>Replication data for: The Constraining Power of International Treaties: Theory and Methods</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E541" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F541" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="542">
@@ -15331,7 +15331,7 @@
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>Thematic map of Massachusetts cities and towns 1999: education, poverty, and income</t>
+          <t>The National Merit Twin Study</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
@@ -15341,11 +15341,11 @@
       </c>
       <c r="E542" t="inlineStr">
         <is>
-          <t>Social work activities without accommodation</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="F542" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="543">
@@ -15359,21 +15359,21 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>Bilateral Trade</t>
+          <t>Thematic map of Massachusetts cities and towns 1999: education, poverty, and income</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
         <is>
-          <t>Water collection, treatment and supply</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E543" t="inlineStr">
         <is>
-          <t>Waste collection, treatment and disposal, and recovery activities</t>
+          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F543" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="544">
@@ -15387,21 +15387,21 @@
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>An Introductory Exploration of Quicklaw-Recorded Citations of Supreme Court of Canada Cases</t>
+          <t>Bilateral Trade</t>
         </is>
       </c>
       <c r="D544" t="inlineStr">
         <is>
-          <t>Printing and reproduction of recorded media</t>
+          <t>Water collection, treatment and supply</t>
         </is>
       </c>
       <c r="E544" t="inlineStr">
         <is>
-          <t>Insurance, reinsurance and pension funding, except compulsory social security</t>
+          <t>Waste collection, treatment and disposal, and recovery activities</t>
         </is>
       </c>
       <c r="F544" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="545">
@@ -15415,21 +15415,21 @@
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>Survey of Income and Program Participation Core and Disability</t>
+          <t>An Introductory Exploration of Quicklaw-Recorded Citations of Supreme Court of Canada Cases</t>
         </is>
       </c>
       <c r="D545" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Printing and reproduction of recorded media</t>
         </is>
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Insurance, reinsurance and pension funding, except compulsory social security</t>
         </is>
       </c>
       <c r="F545" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="546">
@@ -15443,21 +15443,21 @@
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>National Material Capabilities (v3.02)</t>
+          <t>Survey of Income and Program Participation Core and Disability</t>
         </is>
       </c>
       <c r="D546" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="E546" t="inlineStr">
         <is>
-          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F546" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
     </row>
     <row r="547">
@@ -15471,12 +15471,12 @@
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>Replication data for: Presidents and the Politics of Agency Design: Administrative Agency Insulation Event File, 2003</t>
+          <t>National Material Capabilities (v3.02)</t>
         </is>
       </c>
       <c r="D547" t="inlineStr">
         <is>
-          <t>Programming, broadcasting, news agency and other content distribution activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E547" t="inlineStr">
@@ -15485,7 +15485,7 @@
         </is>
       </c>
       <c r="F547" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="548">
@@ -15499,12 +15499,12 @@
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>Towards an Objective Account of Nutrition and Health in Colonial Kenya: A Study of Stature in African Army Recruits and Civilians, 1880–1980</t>
+          <t>Replication data for: Presidents and the Politics of Agency Design: Administrative Agency Insulation Event File, 2003</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Programming, broadcasting, news agency and other content distribution activities</t>
         </is>
       </c>
       <c r="E548" t="inlineStr">
@@ -15513,7 +15513,7 @@
         </is>
       </c>
       <c r="F548" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="549">
@@ -15527,21 +15527,21 @@
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>Other Political Data (updated 2005)</t>
+          <t>Towards an Objective Account of Nutrition and Health in Colonial Kenya: A Study of Stature in African Army Recruits and Civilians, 1880–1980</t>
         </is>
       </c>
       <c r="D549" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>Water collection, treatment and supply</t>
+          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F549" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="550">
@@ -15555,7 +15555,7 @@
       </c>
       <c r="C550" t="inlineStr">
         <is>
-          <t>International Governmental Organization (IGO) Data (v2.1)</t>
+          <t>Other Political Data (updated 2005)</t>
         </is>
       </c>
       <c r="D550" t="inlineStr">
@@ -15565,11 +15565,11 @@
       </c>
       <c r="E550" t="inlineStr">
         <is>
-          <t>Activities of extraterritorial organizations and bodies</t>
+          <t>Water collection, treatment and supply</t>
         </is>
       </c>
       <c r="F550" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="551">
@@ -15583,21 +15583,21 @@
       </c>
       <c r="C551" t="inlineStr">
         <is>
-          <t>Employer Attitudes towards Older Workers, 2006</t>
+          <t>International Governmental Organization (IGO) Data (v2.1)</t>
         </is>
       </c>
       <c r="D551" t="inlineStr">
         <is>
-          <t>Employment activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E551" t="inlineStr">
         <is>
-          <t>Insurance, reinsurance and pension funding, except compulsory social security</t>
+          <t>Activities of extraterritorial organizations and bodies</t>
         </is>
       </c>
       <c r="F551" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="552">
@@ -15611,21 +15611,21 @@
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>Replication data for: No More Wilder Effect, Never a Whitman Effect: When and Why Polls Mislead about Black and Female Candidates</t>
+          <t>Employer Attitudes towards Older Workers, 2006</t>
         </is>
       </c>
       <c r="D552" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Employment activities</t>
         </is>
       </c>
       <c r="E552" t="inlineStr">
         <is>
-          <t>Mining support service activities</t>
+          <t>Insurance, reinsurance and pension funding, except compulsory social security</t>
         </is>
       </c>
       <c r="F552" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="553">
@@ -15639,21 +15639,21 @@
       </c>
       <c r="C553" t="inlineStr">
         <is>
-          <t>Militarized Interstate Disputes (v3.02)</t>
+          <t>Replication data for: No More Wilder Effect, Never a Whitman Effect: When and Why Polls Mislead about Black and Female Candidates</t>
         </is>
       </c>
       <c r="D553" t="inlineStr">
         <is>
-          <t>Activities of membership organizations</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>Mining support service activities</t>
         </is>
       </c>
       <c r="F553" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="554">
@@ -15667,21 +15667,21 @@
       </c>
       <c r="C554" t="inlineStr">
         <is>
-          <t>Controls Data (Geographic, Climatic etc.)</t>
+          <t>Militarized Interstate Disputes (v3.02)</t>
         </is>
       </c>
       <c r="D554" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Activities of membership organizations</t>
         </is>
       </c>
       <c r="E554" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F554" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
     </row>
     <row r="555">
@@ -15695,21 +15695,21 @@
       </c>
       <c r="C555" t="inlineStr">
         <is>
-          <t>Replication data for: State System Membership List, v2004.1</t>
+          <t>Controls Data (Geographic, Climatic etc.)</t>
         </is>
       </c>
       <c r="D555" t="inlineStr">
         <is>
-          <t>Water collection, treatment and supply</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="E555" t="inlineStr">
         <is>
-          <t>Waste collection, treatment and disposal, and recovery activities</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="F555" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="556">
@@ -15723,21 +15723,21 @@
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>Economic Data (updated 2005)</t>
+          <t>Replication data for: State System Membership List, v2004.1</t>
         </is>
       </c>
       <c r="D556" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Water collection, treatment and supply</t>
         </is>
       </c>
       <c r="E556" t="inlineStr">
         <is>
-          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>Waste collection, treatment and disposal, and recovery activities</t>
         </is>
       </c>
       <c r="F556" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="557">
@@ -15751,21 +15751,21 @@
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>Replication data for: The Diversity Discount: When Increasing Ethnic and Racial Diversity Prevents Tax Increases</t>
+          <t>Economic Data (updated 2005)</t>
         </is>
       </c>
       <c r="D557" t="inlineStr">
         <is>
-          <t>Activities of advertising, market research and public relations</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E557" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F557" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="558">
@@ -15779,21 +15779,21 @@
       </c>
       <c r="C558" t="inlineStr">
         <is>
-          <t>Direct Contiguity, 1816-2000 (v3.0)</t>
+          <t>Replication data for: The Diversity Discount: When Increasing Ethnic and Racial Diversity Prevents Tax Increases</t>
         </is>
       </c>
       <c r="D558" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Activities of advertising, market research and public relations</t>
         </is>
       </c>
       <c r="E558" t="inlineStr">
         <is>
-          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="F558" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="559">
@@ -15807,21 +15807,21 @@
       </c>
       <c r="C559" t="inlineStr">
         <is>
-          <t>Replication data for: Peace Time: Cease-Fire Agreements and the Durability of Peace</t>
+          <t>Direct Contiguity, 1816-2000 (v3.0)</t>
         </is>
       </c>
       <c r="D559" t="inlineStr">
         <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
           <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
-      <c r="E559" t="inlineStr">
-        <is>
-          <t>Insurance, reinsurance and pension funding, except compulsory social security</t>
-        </is>
-      </c>
       <c r="F559" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="560">
@@ -15835,7 +15835,7 @@
       </c>
       <c r="C560" t="inlineStr">
         <is>
-          <t>New Violence Data</t>
+          <t>Replication data for: Peace Time: Cease-Fire Agreements and the Durability of Peace</t>
         </is>
       </c>
       <c r="D560" t="inlineStr">
@@ -15849,7 +15849,7 @@
         </is>
       </c>
       <c r="F560" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="561">
@@ -15863,21 +15863,21 @@
       </c>
       <c r="C561" t="inlineStr">
         <is>
-          <t>National Household Education Survey Program (NHES): 2005 Data</t>
+          <t>New Violence Data</t>
         </is>
       </c>
       <c r="D561" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="E561" t="inlineStr">
         <is>
-          <t>Water collection, treatment and supply</t>
+          <t>Insurance, reinsurance and pension funding, except compulsory social security</t>
         </is>
       </c>
       <c r="F561" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
     </row>
     <row r="562">
@@ -15891,21 +15891,21 @@
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>Replication data for: On the Estimation of Disability-Free Life Expectancy: Sullivan's Method and Its Extension</t>
+          <t>National Household Education Survey Program (NHES): 2005 Data</t>
         </is>
       </c>
       <c r="D562" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E562" t="inlineStr">
         <is>
-          <t>Social work activities without accommodation</t>
+          <t>Water collection, treatment and supply</t>
         </is>
       </c>
       <c r="F562" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="563">
@@ -15919,21 +15919,21 @@
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>Alliances (v3.03)</t>
+          <t>Replication data for: On the Estimation of Disability-Free Life Expectancy: Sullivan's Method and Its Extension</t>
         </is>
       </c>
       <c r="D563" t="inlineStr">
         <is>
-          <t>Public administration and defence; compulsory social security</t>
+          <t>Human health activities</t>
         </is>
       </c>
       <c r="E563" t="inlineStr">
         <is>
-          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
+          <t>Social work activities without accommodation</t>
         </is>
       </c>
       <c r="F563" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="564">
@@ -15947,21 +15947,21 @@
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>Peoria GIS Data, 2003</t>
+          <t>Alliances (v3.03)</t>
         </is>
       </c>
       <c r="D564" t="inlineStr">
         <is>
-          <t>Human health activities</t>
+          <t>Public administration and defence; compulsory social security</t>
         </is>
       </c>
       <c r="E564" t="inlineStr">
         <is>
-          <t>Library, archives, museum and other cultural activities</t>
+          <t>Computing infrastructure, data processing, hosting, and other information service activities</t>
         </is>
       </c>
       <c r="F564" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="565">

</xml_diff>